<commit_message>
Updated Output variables; Added additional test cases to cover gaps.
</commit_message>
<xml_diff>
--- a/rules/CORE-000533/positive/01/data/unit-test-coreid-CG0138-positive.xlsx
+++ b/rules/CORE-000533/positive/01/data/unit-test-coreid-CG0138-positive.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="suppdm.xpt" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="suppec.xpt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="relrec.xpt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,6 +549,18 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>Supplemental Qualifiers for Exposure</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Related Records</t>
         </is>
       </c>
     </row>
@@ -1222,4 +1235,216 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STUDYID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>RDOMAIN</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>IDVAR</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>IDVARVAL</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>RELTYPE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>RELID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Study Identifier</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Related Domain Abbreviation</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unique Subject Identifier</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Identifying Variable</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Identifying Variable Value</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Relationship Type</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Relationship Identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CDISC009</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AESEQ</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CDISC009</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CMSEQ</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>